<commit_message>
Atualizando o workspace e arquivos de configuração, incluindo a modificação do título e conteúdo da nota "Estrutura da Planilha FECHAMENTO GERAL 2026 HUGO". Removendo arquivos temporários obsoletos e ajustando referências internas. Adicionando novas notas sobre o mapeamento de colunas ODBC e atualizando a data de última modificação nas notas de análise financeira e controle. Essas alterações visam aprimorar a clareza e a precisão das informações financeiras e operacionais.
</commit_message>
<xml_diff>
--- a/02-Referencias/FOPA/CARGA FOPA - MAI2026.xlsx
+++ b/02-Referencias/FOPA/CARGA FOPA - MAI2026.xlsx
@@ -1,26 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\julio.santana\Documents\Projects\Cofre_Trabalho\02-Referencias\FOPA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C223CAEC-7473-4DF9-AB8E-900CE0D31D08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C65B441F-4C51-495E-9417-0705EDDD86E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="3" xr2:uid="{5AA1821D-7BB5-4576-8642-36CD60D2E92F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{5AA1821D-7BB5-4576-8642-36CD60D2E92F}"/>
   </bookViews>
   <sheets>
-    <sheet name="Base" sheetId="2" r:id="rId1"/>
-    <sheet name="Ajustes" sheetId="3" r:id="rId2"/>
-    <sheet name="TD" sheetId="4" r:id="rId3"/>
-    <sheet name="Base_R" sheetId="5" r:id="rId4"/>
+    <sheet name="Planilha1" sheetId="6" r:id="rId1"/>
+    <sheet name="Base" sheetId="2" r:id="rId2"/>
+    <sheet name="Ajustes" sheetId="3" r:id="rId3"/>
+    <sheet name="TD" sheetId="4" r:id="rId4"/>
+    <sheet name="Base_R" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="515" r:id="rId5"/>
+    <pivotCache cacheId="194" r:id="rId6"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="628" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="890" uniqueCount="185">
   <si>
     <t>CENTRO DE CUSTO</t>
   </si>
@@ -606,8 +607,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -635,13 +644,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1403,7 +1413,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BDE0B441-B84B-4354-B631-06499DF208E4}" name="Tabela dinâmica1" cacheId="515" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{BDE0B441-B84B-4354-B631-06499DF208E4}" name="Tabela dinâmica1" cacheId="194" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B52" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField axis="axisRow" showAll="0">
@@ -2007,6 +2017,1068 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A70AE26B-9FAC-4161-B144-7C8FCA89B2FF}">
+  <dimension ref="A1:B131"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="31.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>16</v>
+      </c>
+      <c r="B16" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>22</v>
+      </c>
+      <c r="B18" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>26</v>
+      </c>
+      <c r="B20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>26</v>
+      </c>
+      <c r="B21" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>29</v>
+      </c>
+      <c r="B23" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+      <c r="B24" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>29</v>
+      </c>
+      <c r="B26" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>29</v>
+      </c>
+      <c r="B28" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
+      <c r="B31" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+      <c r="B32" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>29</v>
+      </c>
+      <c r="B33" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>29</v>
+      </c>
+      <c r="B34" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>29</v>
+      </c>
+      <c r="B36" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>29</v>
+      </c>
+      <c r="B37" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>29</v>
+      </c>
+      <c r="B38" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>29</v>
+      </c>
+      <c r="B39" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>29</v>
+      </c>
+      <c r="B40" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>49</v>
+      </c>
+      <c r="B41" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>49</v>
+      </c>
+      <c r="B42" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>52</v>
+      </c>
+      <c r="B43" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>54</v>
+      </c>
+      <c r="B44" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>54</v>
+      </c>
+      <c r="B45" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>54</v>
+      </c>
+      <c r="B46" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>58</v>
+      </c>
+      <c r="B47" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>60</v>
+      </c>
+      <c r="B48" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>62</v>
+      </c>
+      <c r="B49" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>62</v>
+      </c>
+      <c r="B50" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>65</v>
+      </c>
+      <c r="B51" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>67</v>
+      </c>
+      <c r="B52" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>67</v>
+      </c>
+      <c r="B53" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>67</v>
+      </c>
+      <c r="B54" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>67</v>
+      </c>
+      <c r="B55" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>72</v>
+      </c>
+      <c r="B56" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>72</v>
+      </c>
+      <c r="B57" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>72</v>
+      </c>
+      <c r="B58" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>76</v>
+      </c>
+      <c r="B59" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>78</v>
+      </c>
+      <c r="B60" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>78</v>
+      </c>
+      <c r="B61" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>78</v>
+      </c>
+      <c r="B62" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>78</v>
+      </c>
+      <c r="B63" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>78</v>
+      </c>
+      <c r="B64" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>78</v>
+      </c>
+      <c r="B65" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>85</v>
+      </c>
+      <c r="B66" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>87</v>
+      </c>
+      <c r="B67" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>89</v>
+      </c>
+      <c r="B68" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>89</v>
+      </c>
+      <c r="B69" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>89</v>
+      </c>
+      <c r="B70" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>89</v>
+      </c>
+      <c r="B71" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>94</v>
+      </c>
+      <c r="B72" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>96</v>
+      </c>
+      <c r="B73" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>96</v>
+      </c>
+      <c r="B74" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>96</v>
+      </c>
+      <c r="B75" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>96</v>
+      </c>
+      <c r="B76" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>96</v>
+      </c>
+      <c r="B77" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>96</v>
+      </c>
+      <c r="B78" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>96</v>
+      </c>
+      <c r="B79" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>104</v>
+      </c>
+      <c r="B80" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>104</v>
+      </c>
+      <c r="B81" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>104</v>
+      </c>
+      <c r="B82" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>104</v>
+      </c>
+      <c r="B83" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>109</v>
+      </c>
+      <c r="B84" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>109</v>
+      </c>
+      <c r="B85" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>112</v>
+      </c>
+      <c r="B86" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>112</v>
+      </c>
+      <c r="B87" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>112</v>
+      </c>
+      <c r="B88" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>116</v>
+      </c>
+      <c r="B89" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>116</v>
+      </c>
+      <c r="B90" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>116</v>
+      </c>
+      <c r="B91" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>116</v>
+      </c>
+      <c r="B92" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>116</v>
+      </c>
+      <c r="B93" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>116</v>
+      </c>
+      <c r="B94" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>116</v>
+      </c>
+      <c r="B95" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>124</v>
+      </c>
+      <c r="B96" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>124</v>
+      </c>
+      <c r="B97" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>124</v>
+      </c>
+      <c r="B98" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>128</v>
+      </c>
+      <c r="B99" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>130</v>
+      </c>
+      <c r="B100" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>130</v>
+      </c>
+      <c r="B101" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>133</v>
+      </c>
+      <c r="B102" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>135</v>
+      </c>
+      <c r="B103" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>135</v>
+      </c>
+      <c r="B104" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>135</v>
+      </c>
+      <c r="B105" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>139</v>
+      </c>
+      <c r="B106" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>141</v>
+      </c>
+      <c r="B107" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>141</v>
+      </c>
+      <c r="B108" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>144</v>
+      </c>
+      <c r="B109" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>146</v>
+      </c>
+      <c r="B110" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>146</v>
+      </c>
+      <c r="B111" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>149</v>
+      </c>
+      <c r="B112" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>149</v>
+      </c>
+      <c r="B113" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>152</v>
+      </c>
+      <c r="B114" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>152</v>
+      </c>
+      <c r="B115" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>155</v>
+      </c>
+      <c r="B116" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>157</v>
+      </c>
+      <c r="B117" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>159</v>
+      </c>
+      <c r="B118" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>159</v>
+      </c>
+      <c r="B119" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>162</v>
+      </c>
+      <c r="B120" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>162</v>
+      </c>
+      <c r="B121" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>162</v>
+      </c>
+      <c r="B122" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>166</v>
+      </c>
+      <c r="B123" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>166</v>
+      </c>
+      <c r="B124" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>169</v>
+      </c>
+      <c r="B125" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>169</v>
+      </c>
+      <c r="B126" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>172</v>
+      </c>
+      <c r="B127" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>172</v>
+      </c>
+      <c r="B128" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>172</v>
+      </c>
+      <c r="B129" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>176</v>
+      </c>
+      <c r="B130" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>176</v>
+      </c>
+      <c r="B131" t="s">
+        <v>178</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D3EAF3DB-5B60-44C1-A543-AD857EDB884C}">
   <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3470,7 +4542,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41F654D9-7273-4002-A290-302F287301EF}">
   <dimension ref="A1:C132"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4934,7 +6006,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1ED9253-9B4E-46DB-AEFD-3F2113317E3F}">
   <dimension ref="A3:B52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5348,7 +6420,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD62DB05-89D3-49C1-9636-81F6AC667EA3}">
   <dimension ref="A1:B48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>